<commit_message>
Add hierarchy in holiday
</commit_message>
<xml_diff>
--- a/algo.xlsx
+++ b/algo.xlsx
@@ -887,7 +887,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'state_Vic'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'state_Vic'})</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -940,7 +940,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_type_NoHoliday'})</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1031,7 +1031,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>frozenset({'state_Vic', 'time_of_day_Night'})</t>
+          <t>frozenset({'time_of_day_Night', 'state_Vic'})</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1271,7 +1271,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'vehicle_type_involved_Heavy Vehicle Involved'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'vehicle_type_involved_Heavy Vehicle Involved'})</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1415,7 +1415,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'age_group_65_to_74'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'age_group_65_to_74'})</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1468,7 +1468,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'time_of_day_Day'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_of_day_Day'})</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1511,7 +1511,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'age_group_75_or_older'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'age_group_75_or_older'})</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'time_of_day_Day'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_of_day_Day'})</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1607,7 +1607,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'time_cat_Rush'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_cat_Rush'})</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'time_of_day_Day'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_of_day_Day'})</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1991,7 +1991,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'state_Vic', 'speed_limit_High'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'state_Vic', 'speed_limit_High'})</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_type_NoHoliday'})</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -2183,7 +2183,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'state_Vic', 'speed_limit_Very High'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'speed_limit_Very High', 'state_Vic'})</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2231,12 +2231,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>frozenset({'state_Vic', 'speed_limit_Very High'})</t>
+          <t>frozenset({'speed_limit_Very High', 'state_Vic'})</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_type_NoHoliday'})</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -2423,7 +2423,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'state_Vic', 'time_of_day_Day'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'state_Vic', 'time_of_day_Day'})</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'vehicle_type_involved_No Heavy Vehicle Involved'})</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -2519,7 +2519,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'state_Vic', 'time_of_day_Night'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_of_day_Night', 'state_Vic'})</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2567,12 +2567,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>frozenset({'state_Vic', 'time_of_day_Night'})</t>
+          <t>frozenset({'time_of_day_Night', 'state_Vic'})</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_type_NoHoliday'})</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -2615,7 +2615,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>frozenset({'time_cat_Not Rush', 'state_Vic', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_cat_Not Rush', 'state_Vic'})</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2668,7 +2668,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_type_NoHoliday'})</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -2711,7 +2711,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>frozenset({'state_Vic', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'state_Vic'})</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'time_cat_Not Rush', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'time_cat_Not Rush', 'holiday_type_NoHoliday'})</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -2999,7 +2999,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'age_group_17_to_25', 'speed_limit_High'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'age_group_17_to_25', 'speed_limit_High'})</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3052,7 +3052,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'time_of_day_Night'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_of_day_Night'})</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -3095,7 +3095,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'time_cat_Rush', 'speed_limit_High'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_cat_Rush', 'speed_limit_High'})</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3148,7 +3148,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'time_of_day_Day'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_of_day_Day'})</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -3287,7 +3287,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>frozenset({'age_group_26_to_39', 'speed_limit_High', 'time_cat_Not Rush'})</t>
+          <t>frozenset({'time_cat_Not Rush', 'age_group_26_to_39', 'speed_limit_High'})</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3335,7 +3335,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>frozenset({'speed_limit_Very High', 'time_cat_Rush', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'speed_limit_Very High', 'time_cat_Rush'})</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3388,7 +3388,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'time_of_day_Day'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_of_day_Day'})</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -3431,7 +3431,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>frozenset({'time_cat_Not Rush', 'vehicle_type_involved_Heavy Vehicle Involved', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_cat_Not Rush', 'vehicle_type_involved_Heavy Vehicle Involved'})</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3479,7 +3479,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>frozenset({'time_cat_Not Rush', 'age_group_17_to_25', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_cat_Not Rush', 'age_group_17_to_25'})</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3532,7 +3532,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>frozenset({'time_of_day_Night', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_of_day_Night'})</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -3575,7 +3575,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_NoHoliday', 'age_group_17_to_25'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'age_group_17_to_25', 'holiday_type_NoHoliday'})</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3623,7 +3623,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>frozenset({'time_cat_Not Rush', 'age_group_26_to_39', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'age_group_26_to_39', 'time_cat_Not Rush'})</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3671,7 +3671,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>frozenset({'time_cat_Not Rush', 'holiday_NoHoliday', 'age_group_75_or_older'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_cat_Not Rush', 'age_group_75_or_older'})</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3719,97 +3719,97 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>frozenset({'time_cat_Not Rush', 'age_group_75_or_older'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'age_group_75_or_older'})</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'time_of_day_Day'})</t>
+          <t>frozenset({'time_cat_Not Rush', 'time_of_day_Day'})</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>0.07961458663009459</v>
+        <v>0.09579069522101487</v>
       </c>
       <c r="D69" t="n">
-        <v>0.5481239230579878</v>
+        <v>0.4303372366986672</v>
       </c>
       <c r="E69" t="n">
         <v>0.06368463621338397</v>
       </c>
       <c r="F69" t="n">
-        <v>0.7999116607773852</v>
+        <v>0.6648311306901615</v>
       </c>
       <c r="G69" t="n">
-        <v>1.459362795760987</v>
+        <v>1.544907281996823</v>
       </c>
       <c r="H69" t="n">
         <v>1</v>
       </c>
       <c r="I69" t="n">
-        <v>0.02004597665705649</v>
+        <v>0.0224623331305282</v>
       </c>
       <c r="J69" t="n">
-        <v>2.258382865776414</v>
+        <v>1.699629098831139</v>
       </c>
       <c r="K69" t="n">
-        <v>0.3419974129155443</v>
+        <v>0.3900777866060614</v>
       </c>
       <c r="L69" t="n">
-        <v>0.1129052369077307</v>
+        <v>0.1377133949279495</v>
       </c>
       <c r="M69" t="n">
-        <v>0.5572052838542025</v>
+        <v>0.4116363383706981</v>
       </c>
       <c r="N69" t="n">
-        <v>0.4580491132526177</v>
+        <v>0.4064094366423229</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'age_group_75_or_older'})</t>
+          <t>frozenset({'time_cat_Not Rush', 'age_group_75_or_older'})</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>frozenset({'time_cat_Not Rush', 'time_of_day_Day'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_of_day_Day'})</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>0.09579069522101487</v>
+        <v>0.07961458663009459</v>
       </c>
       <c r="D70" t="n">
-        <v>0.4303372366986672</v>
+        <v>0.5481239230579878</v>
       </c>
       <c r="E70" t="n">
         <v>0.06368463621338397</v>
       </c>
       <c r="F70" t="n">
-        <v>0.6648311306901615</v>
+        <v>0.7999116607773852</v>
       </c>
       <c r="G70" t="n">
-        <v>1.544907281996823</v>
+        <v>1.459362795760987</v>
       </c>
       <c r="H70" t="n">
         <v>1</v>
       </c>
       <c r="I70" t="n">
-        <v>0.0224623331305282</v>
+        <v>0.02004597665705649</v>
       </c>
       <c r="J70" t="n">
-        <v>1.699629098831139</v>
+        <v>2.258382865776414</v>
       </c>
       <c r="K70" t="n">
-        <v>0.3900777866060614</v>
+        <v>0.3419974129155443</v>
       </c>
       <c r="L70" t="n">
-        <v>0.1377133949279495</v>
+        <v>0.1129052369077307</v>
       </c>
       <c r="M70" t="n">
-        <v>0.4116363383706981</v>
+        <v>0.5572052838542025</v>
       </c>
       <c r="N70" t="n">
-        <v>0.4064094366423229</v>
+        <v>0.4580491132526177</v>
       </c>
     </row>
     <row r="71">
@@ -3820,7 +3820,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>frozenset({'time_cat_Not Rush', 'time_of_day_Day', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_cat_Not Rush', 'time_of_day_Day'})</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -3863,7 +3863,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_NoHoliday', 'time_cat_Rush'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_cat_Rush', 'vehicle_type_involved_No Heavy Vehicle Involved'})</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3916,7 +3916,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'time_of_day_Day'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_of_day_Day'})</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -4007,7 +4007,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'time_cat_Not Rush', 'age_group_26_to_39'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'age_group_26_to_39', 'time_cat_Not Rush'})</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -4055,7 +4055,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'state_Vic', 'speed_limit_High', 'time_cat_Not Rush'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_cat_Not Rush', 'state_Vic', 'speed_limit_High'})</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4103,97 +4103,97 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'state_Vic', 'speed_limit_High'})</t>
+          <t>frozenset({'time_cat_Not Rush', 'state_Vic', 'speed_limit_High'})</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'time_cat_Not Rush'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_type_NoHoliday'})</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>0.09373351619369132</v>
+        <v>0.08397510285895136</v>
       </c>
       <c r="D77" t="n">
-        <v>0.4600872103245771</v>
+        <v>0.5126947286985266</v>
       </c>
       <c r="E77" t="n">
         <v>0.07259907866511939</v>
       </c>
       <c r="F77" t="n">
-        <v>0.7745263552804352</v>
+        <v>0.8645309882747069</v>
       </c>
       <c r="G77" t="n">
-        <v>1.683433787985611</v>
+        <v>1.686249028675046</v>
       </c>
       <c r="H77" t="n">
         <v>1</v>
       </c>
       <c r="I77" t="n">
-        <v>0.02947348668565038</v>
+        <v>0.02954548608741845</v>
       </c>
       <c r="J77" t="n">
-        <v>2.394571615440666</v>
+        <v>3.597171523548434</v>
       </c>
       <c r="K77" t="n">
-        <v>0.4479654166911415</v>
+        <v>0.4442758970902324</v>
       </c>
       <c r="L77" t="n">
-        <v>0.1508641163360006</v>
+        <v>0.1385291552036503</v>
       </c>
       <c r="M77" t="n">
-        <v>0.5823887690174707</v>
+        <v>0.7220038039738653</v>
       </c>
       <c r="N77" t="n">
-        <v>0.4661602617537958</v>
+        <v>0.5030669619517504</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>frozenset({'time_cat_Not Rush', 'state_Vic', 'speed_limit_High'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'state_Vic', 'speed_limit_High'})</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'time_cat_Not Rush'})</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>0.08397510285895136</v>
+        <v>0.09373351619369132</v>
       </c>
       <c r="D78" t="n">
-        <v>0.5126947286985266</v>
+        <v>0.4600872103245771</v>
       </c>
       <c r="E78" t="n">
         <v>0.07259907866511939</v>
       </c>
       <c r="F78" t="n">
-        <v>0.8645309882747069</v>
+        <v>0.7745263552804352</v>
       </c>
       <c r="G78" t="n">
-        <v>1.686249028675046</v>
+        <v>1.683433787985611</v>
       </c>
       <c r="H78" t="n">
         <v>1</v>
       </c>
       <c r="I78" t="n">
-        <v>0.02954548608741845</v>
+        <v>0.02947348668565038</v>
       </c>
       <c r="J78" t="n">
-        <v>3.597171523548434</v>
+        <v>2.394571615440666</v>
       </c>
       <c r="K78" t="n">
-        <v>0.4442758970902324</v>
+        <v>0.4479654166911415</v>
       </c>
       <c r="L78" t="n">
-        <v>0.1385291552036503</v>
+        <v>0.1508641163360006</v>
       </c>
       <c r="M78" t="n">
-        <v>0.7220038039738653</v>
+        <v>0.5823887690174707</v>
       </c>
       <c r="N78" t="n">
-        <v>0.5030669619517504</v>
+        <v>0.4661602617537958</v>
       </c>
     </row>
     <row r="79">
@@ -4204,7 +4204,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_NoHoliday', 'time_cat_Not Rush'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'time_cat_Not Rush', 'holiday_type_NoHoliday'})</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -4247,7 +4247,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>frozenset({'speed_limit_Very High', 'state_Vic', 'time_cat_Not Rush', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'speed_limit_Very High', 'state_Vic', 'time_cat_Not Rush'})</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4295,97 +4295,97 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>frozenset({'speed_limit_Very High', 'state_Vic', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'speed_limit_Very High', 'state_Vic', 'time_cat_Not Rush'})</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'time_cat_Not Rush'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_type_NoHoliday'})</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>0.1024193831979463</v>
+        <v>0.09058620810915356</v>
       </c>
       <c r="D81" t="n">
-        <v>0.4600872103245771</v>
+        <v>0.5126947286985266</v>
       </c>
       <c r="E81" t="n">
         <v>0.07099905053275662</v>
       </c>
       <c r="F81" t="n">
-        <v>0.6932188841201716</v>
+        <v>0.783773291925466</v>
       </c>
       <c r="G81" t="n">
-        <v>1.506711920183844</v>
+        <v>1.528732885385951</v>
       </c>
       <c r="H81" t="n">
         <v>1</v>
       </c>
       <c r="I81" t="n">
-        <v>0.02387720223404963</v>
+        <v>0.02455597914240587</v>
       </c>
       <c r="J81" t="n">
-        <v>1.759928371493754</v>
+        <v>2.253677520417587</v>
       </c>
       <c r="K81" t="n">
-        <v>0.3746773426547197</v>
+        <v>0.3803147581445584</v>
       </c>
       <c r="L81" t="n">
-        <v>0.1444515990555914</v>
+        <v>0.1333861857100387</v>
       </c>
       <c r="M81" t="n">
-        <v>0.4317950570049384</v>
+        <v>0.5562807939732618</v>
       </c>
       <c r="N81" t="n">
-        <v>0.4237676948211971</v>
+        <v>0.4611277036121723</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>frozenset({'speed_limit_Very High', 'state_Vic', 'time_cat_Not Rush'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'speed_limit_Very High', 'state_Vic'})</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'time_cat_Not Rush'})</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>0.09058620810915356</v>
+        <v>0.1024193831979463</v>
       </c>
       <c r="D82" t="n">
-        <v>0.5126947286985266</v>
+        <v>0.4600872103245771</v>
       </c>
       <c r="E82" t="n">
         <v>0.07099905053275662</v>
       </c>
       <c r="F82" t="n">
-        <v>0.783773291925466</v>
+        <v>0.6932188841201716</v>
       </c>
       <c r="G82" t="n">
-        <v>1.528732885385951</v>
+        <v>1.506711920183844</v>
       </c>
       <c r="H82" t="n">
         <v>1</v>
       </c>
       <c r="I82" t="n">
-        <v>0.02455597914240587</v>
+        <v>0.02387720223404963</v>
       </c>
       <c r="J82" t="n">
-        <v>2.253677520417587</v>
+        <v>1.759928371493754</v>
       </c>
       <c r="K82" t="n">
-        <v>0.3803147581445584</v>
+        <v>0.3746773426547197</v>
       </c>
       <c r="L82" t="n">
-        <v>0.1333861857100387</v>
+        <v>0.1444515990555914</v>
       </c>
       <c r="M82" t="n">
-        <v>0.5562807939732618</v>
+        <v>0.4317950570049384</v>
       </c>
       <c r="N82" t="n">
-        <v>0.4611277036121723</v>
+        <v>0.4237676948211971</v>
       </c>
     </row>
     <row r="83">
@@ -4396,7 +4396,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_NoHoliday', 'time_cat_Not Rush'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'time_cat_Not Rush', 'holiday_type_NoHoliday'})</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -4439,7 +4439,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'state_Vic', 'time_cat_Not Rush', 'time_of_day_Day'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_cat_Not Rush', 'state_Vic', 'time_of_day_Day'})</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4487,103 +4487,103 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'state_Vic', 'time_of_day_Day'})</t>
+          <t>frozenset({'time_cat_Not Rush', 'state_Vic', 'time_of_day_Day'})</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'time_cat_Not Rush'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_type_NoHoliday'})</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>0.1175756936385695</v>
+        <v>0.09248514259591377</v>
       </c>
       <c r="D85" t="n">
-        <v>0.4600872103245771</v>
+        <v>0.5126947286985266</v>
       </c>
       <c r="E85" t="n">
         <v>0.07247599957801455</v>
       </c>
       <c r="F85" t="n">
-        <v>0.6164199192462987</v>
+        <v>0.7836501901140684</v>
       </c>
       <c r="G85" t="n">
-        <v>1.339789295189131</v>
+        <v>1.528492777960408</v>
       </c>
       <c r="H85" t="n">
         <v>1</v>
       </c>
       <c r="I85" t="n">
-        <v>0.01838092668986799</v>
+        <v>0.02505935448615799</v>
       </c>
       <c r="J85" t="n">
-        <v>1.407562114838032</v>
+        <v>2.252395190725615</v>
       </c>
       <c r="K85" t="n">
-        <v>0.2874059315104739</v>
+        <v>0.3809973210800953</v>
       </c>
       <c r="L85" t="n">
-        <v>0.1434637338159543</v>
+        <v>0.1360530745618378</v>
       </c>
       <c r="M85" t="n">
-        <v>0.2895517793081054</v>
+        <v>0.5560281765306703</v>
       </c>
       <c r="N85" t="n">
-        <v>0.3869732874788455</v>
+        <v>0.4625065313202805</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>frozenset({'time_cat_Not Rush', 'state_Vic', 'time_of_day_Day'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'state_Vic', 'time_of_day_Day'})</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'time_cat_Not Rush'})</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>0.09248514259591377</v>
+        <v>0.1175756936385695</v>
       </c>
       <c r="D86" t="n">
-        <v>0.5126947286985266</v>
+        <v>0.4600872103245771</v>
       </c>
       <c r="E86" t="n">
         <v>0.07247599957801455</v>
       </c>
       <c r="F86" t="n">
-        <v>0.7836501901140684</v>
+        <v>0.6164199192462987</v>
       </c>
       <c r="G86" t="n">
-        <v>1.528492777960408</v>
+        <v>1.339789295189131</v>
       </c>
       <c r="H86" t="n">
         <v>1</v>
       </c>
       <c r="I86" t="n">
-        <v>0.02505935448615799</v>
+        <v>0.01838092668986799</v>
       </c>
       <c r="J86" t="n">
-        <v>2.252395190725615</v>
+        <v>1.407562114838032</v>
       </c>
       <c r="K86" t="n">
-        <v>0.3809973210800953</v>
+        <v>0.2874059315104739</v>
       </c>
       <c r="L86" t="n">
-        <v>0.1360530745618378</v>
+        <v>0.1434637338159543</v>
       </c>
       <c r="M86" t="n">
-        <v>0.5560281765306703</v>
+        <v>0.2895517793081054</v>
       </c>
       <c r="N86" t="n">
-        <v>0.4625065313202805</v>
+        <v>0.3869732874788455</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'state_Vic', 'time_of_day_Night', 'time_cat_Not Rush'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_of_day_Night', 'state_Vic', 'time_cat_Not Rush'})</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4631,97 +4631,97 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'state_Vic', 'time_of_day_Night'})</t>
+          <t>frozenset({'time_of_day_Night', 'state_Vic', 'time_cat_Not Rush'})</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'time_cat_Not Rush'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_type_NoHoliday'})</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>0.09236206350880895</v>
+        <v>0.09443682526286176</v>
       </c>
       <c r="D88" t="n">
-        <v>0.4600872103245771</v>
+        <v>0.5126947286985266</v>
       </c>
       <c r="E88" t="n">
         <v>0.08147835566339628</v>
       </c>
       <c r="F88" t="n">
-        <v>0.8821625737673711</v>
+        <v>0.8627816049152859</v>
       </c>
       <c r="G88" t="n">
-        <v>1.917381213759524</v>
+        <v>1.682836894199114</v>
       </c>
       <c r="H88" t="n">
         <v>1</v>
       </c>
       <c r="I88" t="n">
-        <v>0.03898375152380695</v>
+        <v>0.03306109315610321</v>
       </c>
       <c r="J88" t="n">
-        <v>4.581844724014535</v>
+        <v>3.55131154974249</v>
       </c>
       <c r="K88" t="n">
-        <v>0.5271433530215832</v>
+        <v>0.4480806608086847</v>
       </c>
       <c r="L88" t="n">
-        <v>0.1730008213245726</v>
+        <v>0.155004013914905</v>
       </c>
       <c r="M88" t="n">
-        <v>0.7817472960707806</v>
+        <v>0.7184138913206556</v>
       </c>
       <c r="N88" t="n">
-        <v>0.5296279296016126</v>
+        <v>0.5108516893193323</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>frozenset({'time_of_day_Night', 'state_Vic', 'time_cat_Not Rush'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_of_day_Night', 'state_Vic'})</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'time_cat_Not Rush'})</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>0.09443682526286176</v>
+        <v>0.09236206350880895</v>
       </c>
       <c r="D89" t="n">
-        <v>0.5126947286985266</v>
+        <v>0.4600872103245771</v>
       </c>
       <c r="E89" t="n">
         <v>0.08147835566339628</v>
       </c>
       <c r="F89" t="n">
-        <v>0.8627816049152859</v>
+        <v>0.8821625737673711</v>
       </c>
       <c r="G89" t="n">
-        <v>1.682836894199114</v>
+        <v>1.917381213759524</v>
       </c>
       <c r="H89" t="n">
         <v>1</v>
       </c>
       <c r="I89" t="n">
-        <v>0.03306109315610321</v>
+        <v>0.03898375152380695</v>
       </c>
       <c r="J89" t="n">
-        <v>3.55131154974249</v>
+        <v>4.581844724014535</v>
       </c>
       <c r="K89" t="n">
-        <v>0.4480806608086847</v>
+        <v>0.5271433530215832</v>
       </c>
       <c r="L89" t="n">
-        <v>0.155004013914905</v>
+        <v>0.1730008213245726</v>
       </c>
       <c r="M89" t="n">
-        <v>0.7184138913206556</v>
+        <v>0.7817472960707806</v>
       </c>
       <c r="N89" t="n">
-        <v>0.5108516893193323</v>
+        <v>0.5296279296016126</v>
       </c>
     </row>
     <row r="90">
@@ -4732,7 +4732,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_NoHoliday', 'time_cat_Not Rush'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'time_cat_Not Rush', 'holiday_type_NoHoliday'})</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -4775,7 +4775,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'age_group_17_to_25', 'speed_limit_High', 'time_cat_Not Rush'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_cat_Not Rush', 'age_group_17_to_25', 'speed_limit_High'})</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4823,97 +4823,97 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'age_group_17_to_25', 'speed_limit_High'})</t>
+          <t>frozenset({'time_cat_Not Rush', 'age_group_17_to_25', 'speed_limit_High'})</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>frozenset({'time_of_day_Night', 'time_cat_Not Rush'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_of_day_Night'})</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>0.1089425748145022</v>
+        <v>0.101047930513064</v>
       </c>
       <c r="D92" t="n">
-        <v>0.4168512852973239</v>
+        <v>0.4139325526602666</v>
       </c>
       <c r="E92" t="n">
         <v>0.07027815873685692</v>
       </c>
       <c r="F92" t="n">
-        <v>0.645093608779858</v>
+        <v>0.6954933008526188</v>
       </c>
       <c r="G92" t="n">
-        <v>1.547538970210294</v>
+        <v>1.680209242744535</v>
       </c>
       <c r="H92" t="n">
         <v>1</v>
       </c>
       <c r="I92" t="n">
-        <v>0.02486530640183179</v>
+        <v>0.02845113091854711</v>
       </c>
       <c r="J92" t="n">
-        <v>1.643105700908496</v>
+        <v>1.924645497063685</v>
       </c>
       <c r="K92" t="n">
-        <v>0.3970706136473187</v>
+        <v>0.4503421769977219</v>
       </c>
       <c r="L92" t="n">
-        <v>0.1542826263172116</v>
+        <v>0.1580341609995256</v>
       </c>
       <c r="M92" t="n">
-        <v>0.3913964272370995</v>
+        <v>0.4804237967326246</v>
       </c>
       <c r="N92" t="n">
-        <v>0.4068432444101753</v>
+        <v>0.4326374838304382</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>frozenset({'time_cat_Not Rush', 'age_group_17_to_25', 'speed_limit_High'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'age_group_17_to_25', 'speed_limit_High'})</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'time_of_day_Night'})</t>
+          <t>frozenset({'time_of_day_Night', 'time_cat_Not Rush'})</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>0.101047930513064</v>
+        <v>0.1089425748145022</v>
       </c>
       <c r="D93" t="n">
-        <v>0.4139325526602666</v>
+        <v>0.4168512852973239</v>
       </c>
       <c r="E93" t="n">
         <v>0.07027815873685692</v>
       </c>
       <c r="F93" t="n">
-        <v>0.6954933008526188</v>
+        <v>0.645093608779858</v>
       </c>
       <c r="G93" t="n">
-        <v>1.680209242744535</v>
+        <v>1.547538970210294</v>
       </c>
       <c r="H93" t="n">
         <v>1</v>
       </c>
       <c r="I93" t="n">
-        <v>0.02845113091854711</v>
+        <v>0.02486530640183179</v>
       </c>
       <c r="J93" t="n">
-        <v>1.924645497063685</v>
+        <v>1.643105700908496</v>
       </c>
       <c r="K93" t="n">
-        <v>0.4503421769977219</v>
+        <v>0.3970706136473187</v>
       </c>
       <c r="L93" t="n">
-        <v>0.1580341609995256</v>
+        <v>0.1542826263172116</v>
       </c>
       <c r="M93" t="n">
-        <v>0.4804237967326246</v>
+        <v>0.3913964272370995</v>
       </c>
       <c r="N93" t="n">
-        <v>0.4326374838304382</v>
+        <v>0.4068432444101753</v>
       </c>
     </row>
     <row r="94">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'time_of_day_Night', 'time_cat_Not Rush'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_of_day_Night', 'time_cat_Not Rush'})</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -4967,7 +4967,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'holiday_NoHoliday', 'age_group_17_to_25', 'time_cat_Not Rush'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'time_cat_Not Rush', 'age_group_17_to_25', 'holiday_type_NoHoliday'})</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -5020,7 +5020,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>frozenset({'holiday_NoHoliday', 'time_of_day_Night'})</t>
+          <t>frozenset({'holiday_type_NoHoliday', 'time_of_day_Night'})</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -5063,7 +5063,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'age_group_26_to_39', 'time_cat_Not Rush', 'holiday_NoHoliday'})</t>
+          <t>frozenset({'vehicle_type_involved_No Heavy Vehicle Involved', 'age_group_26_to_39', 'time_cat_Not Rush', 'holiday_type_NoHoliday'})</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">

</xml_diff>